<commit_message>
pnr status check module added
</commit_message>
<xml_diff>
--- a/AutomationMavenProject_RedBus/src/test/resources/testdata/TrainTestData.xlsx
+++ b/AutomationMavenProject_RedBus/src/test/resources/testdata/TrainTestData.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\cg_training\Sprint\DAY4\AutomationMavenProject\AutomationMavenProject_RedBus\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\cg_training\Sprint\DAY5\AutomationMavenProject\AutomationMavenProject_RedBus\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560B93C3-53AD-4C11-8B11-A90736B2CACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{360B4C6E-3831-4553-AC10-9EDA2B470C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{3A6A8E8A-8660-494D-BCD0-7A1F7E35A034}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{3A6A8E8A-8660-494D-BCD0-7A1F7E35A034}"/>
   </bookViews>
   <sheets>
     <sheet name="TrainSearchData" sheetId="1" r:id="rId1"/>
+    <sheet name="PNR_Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>trainInput</t>
   </si>
@@ -88,6 +89,39 @@
   </si>
   <si>
     <t>Non-existent name</t>
+  </si>
+  <si>
+    <t>PNR</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>valid</t>
+  </si>
+  <si>
+    <t>Valid PNR - should show details</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>Invalid PNR - should show error</t>
+  </si>
+  <si>
+    <t>short</t>
+  </si>
+  <si>
+    <t>Less than 10 digits</t>
+  </si>
+  <si>
+    <t>long</t>
+  </si>
+  <si>
+    <t>More than 10 digits</t>
   </si>
 </sst>
 </file>
@@ -540,4 +574,73 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4981A902-2C91-4045-91AA-080834EC2A7A}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="3" max="3" width="33.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>6700914458</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>3476986918</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>12345</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>1234567890123</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>